<commit_message>
update roads_data.xlsx: Airport Wadi KPI/trees, Qassim Road trees to plant
</commit_message>
<xml_diff>
--- a/roads_data.xlsx
+++ b/roads_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed\Downloads\Aa_Canopy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FCCC3C5-BCE3-49C9-9A49-4ACA016FF9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7F61AD-8702-4253-81BC-EC301AFD4EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7AAB8FE-2C25-4993-9707-1AE9B1428E4B}"/>
   </bookViews>
@@ -92,9 +92,6 @@
     <t>Trees to be planted to reach planned KPI</t>
   </si>
   <si>
-    <t>Roads</t>
-  </si>
-  <si>
     <t>Airport Road</t>
   </si>
   <si>
@@ -159,6 +156,9 @@
   </si>
   <si>
     <t>Branch of Wadi Al Laysan Phase 2 (KACST)</t>
+  </si>
+  <si>
+    <t>Road</t>
   </si>
 </sst>
 </file>
@@ -169,7 +169,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,14 +178,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -238,7 +230,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -281,10 +273,8 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -296,53 +286,10 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -372,11 +319,26 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -388,11 +350,13 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="thin">
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -401,13 +365,11 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -416,7 +378,9 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -424,8 +388,12 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -433,15 +401,22 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -454,36 +429,8 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -498,9 +445,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -513,9 +458,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -526,9 +469,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -536,102 +477,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="52">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -644,16 +558,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -664,6 +568,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -684,6 +598,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -694,41 +648,411 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1085,770 +1409,770 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="O1" s="21" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="20"/>
+      <c r="A2" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="4">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3">
         <v>5339843</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>3105072</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>19360</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>288353</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>1086200</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>2018871</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>10853</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>30243</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="3">
         <v>1396924</v>
       </c>
-      <c r="K3" s="11">
+      <c r="K3" s="7">
         <v>12</v>
       </c>
-      <c r="L3" s="7">
+      <c r="L3" s="5">
         <v>5.4000276787163966</v>
       </c>
-      <c r="M3" s="7">
+      <c r="M3" s="5">
         <v>20.34142202308195</v>
       </c>
-      <c r="N3" s="12">
+      <c r="N3" s="8">
         <v>46.501816626443883</v>
       </c>
-      <c r="O3" s="16">
+      <c r="O3" s="24">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="5">
+        <v>16</v>
+      </c>
+      <c r="B4" s="4">
         <v>3503507</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>2196951</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>7508</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>3203</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>588536</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>1608415</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>11308</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="3">
         <v>18816</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>1124890</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="9">
         <v>12</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="6">
         <v>9.1422680188736602E-2</v>
       </c>
-      <c r="M4" s="8">
+      <c r="M4" s="6">
         <v>16.79848220654333</v>
       </c>
-      <c r="N4" s="14">
+      <c r="N4" s="10">
         <v>48.906024734644461</v>
       </c>
-      <c r="O4" s="17">
+      <c r="O4" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="5">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4">
         <v>1858085</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>799865</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>3168</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>12986</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>197600</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <v>602265</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="3">
         <v>3875</v>
       </c>
-      <c r="I5" s="4">
+      <c r="I5" s="3">
         <v>7043</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="3">
         <v>414882</v>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="11">
         <v>12</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="6">
         <v>0.69889160076099854</v>
       </c>
-      <c r="M5" s="8">
+      <c r="M5" s="6">
         <v>10.634604983087426</v>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="10">
         <v>32.963077577182958</v>
       </c>
-      <c r="O5" s="17">
+      <c r="O5" s="13">
         <v>406.74490688259107</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="5">
+        <v>18</v>
+      </c>
+      <c r="B6" s="4">
         <v>3612799</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>1285169</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>10558</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>107102</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>467496</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>817673</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>5160</v>
       </c>
-      <c r="I6" s="4">
+      <c r="I6" s="3">
         <v>15718</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>522325</v>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="11">
         <v>12</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="6">
         <v>2.964515878132163</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="6">
         <v>12.939994724312092</v>
       </c>
-      <c r="N6" s="14">
+      <c r="N6" s="10">
         <v>27.397621622459486</v>
       </c>
-      <c r="O6" s="17">
+      <c r="O6" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="5">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4">
         <v>450056</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>144911</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>1516</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>14702</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>82945</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <v>61966</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="3">
         <v>363</v>
       </c>
-      <c r="I7" s="4">
+      <c r="I7" s="3">
         <v>1879</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="3">
         <v>50040</v>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="11">
         <v>12</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="6">
         <v>3.2667045878735088</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="6">
         <v>18.429928719981511</v>
       </c>
-      <c r="N7" s="14">
+      <c r="N7" s="10">
         <v>29.548545069946851</v>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="5">
+        <v>20</v>
+      </c>
+      <c r="B8" s="4">
         <v>2322528</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>739346</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>1059</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>1371</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>62539</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <v>676807</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="3">
         <v>4893</v>
       </c>
-      <c r="I8" s="4">
+      <c r="I8" s="3">
         <v>5952</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="3">
         <v>499072</v>
       </c>
-      <c r="K8" s="15">
+      <c r="K8" s="11">
         <v>12</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="6">
         <v>5.9030504691439674E-2</v>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="6">
         <v>2.6927124237038265</v>
       </c>
-      <c r="N8" s="14">
+      <c r="N8" s="10">
         <v>24.181021714269971</v>
       </c>
-      <c r="O8" s="17">
+      <c r="O8" s="13">
         <v>3660.4048232303044</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="5">
+        <v>21</v>
+      </c>
+      <c r="B9" s="4">
         <v>567004</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>63865</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>583</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>8174</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>21608</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>42257</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>325</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="3">
         <v>908</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="3">
         <v>28499</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="11">
         <v>15</v>
       </c>
-      <c r="L9" s="8">
+      <c r="L9" s="6">
         <v>1.4416124048507595</v>
       </c>
-      <c r="M9" s="8">
+      <c r="M9" s="6">
         <v>3.8109078595565467</v>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="10">
         <v>8.8371510606627126</v>
       </c>
-      <c r="O9" s="17">
+      <c r="O9" s="13">
         <v>1711.728794890781</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="5">
+        <v>22</v>
+      </c>
+      <c r="B10" s="4">
         <v>2098017</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>725672</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>5806</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>95034</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>309776</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>415896</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="3">
         <v>2252</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I10" s="3">
         <v>8058</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="3">
         <v>267634</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="11">
         <v>15</v>
       </c>
-      <c r="L10" s="8">
+      <c r="L10" s="6">
         <v>4.5297059080074185</v>
       </c>
-      <c r="M10" s="8">
+      <c r="M10" s="6">
         <v>14.76518064438944</v>
       </c>
-      <c r="N10" s="14">
+      <c r="N10" s="10">
         <v>27.521702636346607</v>
       </c>
-      <c r="O10" s="17">
+      <c r="O10" s="13">
         <v>92.336234246681357</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="5">
+        <v>23</v>
+      </c>
+      <c r="B11" s="4">
         <v>1664978</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>584392</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>4005</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>38978</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>197462</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>386930</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>2056</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I11" s="3">
         <v>6061</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="3">
         <v>317712</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="11">
         <v>15</v>
       </c>
-      <c r="L11" s="8">
+      <c r="L11" s="6">
         <v>2.3410519538396302</v>
       </c>
-      <c r="M11" s="8">
+      <c r="M11" s="6">
         <v>11.859736284803763</v>
       </c>
-      <c r="N11" s="14">
+      <c r="N11" s="10">
         <v>30.941790221852781</v>
       </c>
-      <c r="O11" s="17">
+      <c r="O11" s="13">
         <v>1060.4583337553556</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="5">
+        <v>24</v>
+      </c>
+      <c r="B12" s="4">
         <v>1495231</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>314326</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>2288</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>33528</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>105263</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>209063</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>1581</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I12" s="3">
         <v>3869</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="3">
         <v>168335</v>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="11">
         <v>15</v>
       </c>
-      <c r="L12" s="8">
+      <c r="L12" s="6">
         <v>2.2423291116890969</v>
       </c>
-      <c r="M12" s="8">
+      <c r="M12" s="6">
         <v>7.039915571573891</v>
       </c>
-      <c r="N12" s="14">
+      <c r="N12" s="10">
         <v>18.298042242302362</v>
       </c>
-      <c r="O12" s="17">
+      <c r="O12" s="13">
         <v>2587.0584649876973</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="5">
+        <v>25</v>
+      </c>
+      <c r="B13" s="4">
         <v>1168715</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>196100</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>3110</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>29624</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>126697</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>69403</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>497</v>
       </c>
-      <c r="I13" s="4">
+      <c r="I13" s="3">
         <v>3607</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="3">
         <v>45784</v>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="11">
         <v>12</v>
       </c>
-      <c r="L13" s="8">
+      <c r="L13" s="6">
         <v>2.5347497037344433</v>
       </c>
-      <c r="M13" s="8">
+      <c r="M13" s="6">
         <v>10.840709668310923</v>
       </c>
-      <c r="N13" s="14">
+      <c r="N13" s="10">
         <v>14.75817457635095</v>
       </c>
-      <c r="O13" s="17">
+      <c r="O13" s="13">
         <v>332.57905080625403</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="5">
+        <v>26</v>
+      </c>
+      <c r="B14" s="4">
         <v>290518</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>39999</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>0</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>0</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>0</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>39999</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="3">
         <v>732</v>
       </c>
-      <c r="I14" s="4">
+      <c r="I14" s="3">
         <v>732</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="3">
         <v>20664</v>
       </c>
-      <c r="K14" s="15">
+      <c r="K14" s="11">
         <v>12</v>
       </c>
-      <c r="L14" s="8">
+      <c r="L14" s="6">
         <v>0</v>
       </c>
-      <c r="M14" s="8">
+      <c r="M14" s="6">
         <v>0</v>
       </c>
-      <c r="N14" s="14">
+      <c r="N14" s="10">
         <v>7.1128122870183601</v>
       </c>
-      <c r="O14" s="17">
-        <v>629.84387173664663</v>
+      <c r="O14" s="13">
+        <v>633.85745454545452</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="5">
+        <v>27</v>
+      </c>
+      <c r="B15" s="4">
         <v>2409239</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>1166044</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>1360</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>4689</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>117471</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <v>1048573</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="3">
         <v>8430</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I15" s="3">
         <v>9790</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="3">
         <v>652419</v>
       </c>
-      <c r="K15" s="15">
+      <c r="K15" s="11">
         <v>12</v>
       </c>
-      <c r="L15" s="8">
+      <c r="L15" s="6">
         <v>0.19462577187236302</v>
       </c>
-      <c r="M15" s="8">
+      <c r="M15" s="6">
         <v>4.8758549898951493</v>
       </c>
-      <c r="N15" s="14">
+      <c r="N15" s="10">
         <v>31.955733739990094</v>
       </c>
-      <c r="O15" s="17">
+      <c r="O15" s="13">
         <v>1987.1052838572923</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="5">
+        <v>28</v>
+      </c>
+      <c r="B16" s="4">
         <v>3469847</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>1184771</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>2940</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>77622</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="3">
         <v>171846</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="3">
         <v>1012926</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="3">
         <v>8307</v>
       </c>
-      <c r="I16" s="4">
+      <c r="I16" s="3">
         <v>11247</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="3">
         <v>650917</v>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="11">
         <v>12</v>
       </c>
-      <c r="L16" s="8">
+      <c r="L16" s="6">
         <v>2.2370438811855395</v>
       </c>
-      <c r="M16" s="8">
+      <c r="M16" s="6">
         <v>4.9525526629848526</v>
       </c>
-      <c r="N16" s="14">
+      <c r="N16" s="10">
         <v>23.711794785187937</v>
       </c>
-      <c r="O16" s="17">
+      <c r="O16" s="13">
         <v>4183.5991620404311</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="5">
+      <c r="A17" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="14">
         <v>2610463</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="26">
         <v>900928</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="26">
         <v>1131</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="26">
         <v>28105</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="26">
         <v>55079</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="26">
         <v>845849</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="26">
         <v>7197</v>
       </c>
-      <c r="I17" s="4">
+      <c r="I17" s="26">
         <v>8328</v>
       </c>
-      <c r="J17" s="4">
+      <c r="J17" s="26">
         <v>564240</v>
       </c>
-      <c r="K17" s="15">
+      <c r="K17" s="27">
         <v>12</v>
       </c>
-      <c r="L17" s="8">
+      <c r="L17" s="15">
         <v>1.0766289351735687</v>
       </c>
-      <c r="M17" s="8">
+      <c r="M17" s="15">
         <v>2.1099322227512896</v>
       </c>
-      <c r="N17" s="14">
+      <c r="N17" s="16">
         <v>23.724488720966356</v>
       </c>
       <c r="O17" s="17">
@@ -1856,311 +2180,307 @@
       </c>
     </row>
     <row r="18" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
+      <c r="A18" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="24">
+      <c r="A19" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="29">
         <v>9298927</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="29">
         <v>8673006</v>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="29">
         <v>679</v>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="29">
         <v>6296</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="29">
         <v>49062</v>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="29">
         <v>8623944</v>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="29">
         <v>58495</v>
       </c>
-      <c r="I19" s="24">
+      <c r="I19" s="29">
         <v>59174</v>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="29">
         <v>4666380</v>
       </c>
-      <c r="K19" s="25">
-        <v>30</v>
-      </c>
-      <c r="L19" s="26">
+      <c r="K19" s="7">
+        <v>7</v>
+      </c>
+      <c r="L19" s="5">
         <v>6.7706736486908642E-2</v>
       </c>
-      <c r="M19" s="26">
+      <c r="M19" s="5">
         <v>0.52760926072438252</v>
       </c>
-      <c r="N19" s="27">
+      <c r="N19" s="8">
         <v>50.709528099317261</v>
       </c>
-      <c r="O19" s="28">
-        <v>37929.116870490398</v>
+      <c r="O19" s="24">
+        <v>8329.5606031144252</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="5">
+      <c r="A20" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="4">
         <v>663931</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="4">
         <v>663931</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="4">
         <v>6405</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="4">
         <v>22994</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="4">
         <v>316287</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="4">
         <v>347643</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="4">
         <v>1286</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="4">
         <v>7691</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="4">
         <v>212371</v>
       </c>
-      <c r="K20" s="13">
+      <c r="K20" s="9">
         <v>30</v>
       </c>
-      <c r="L20" s="8">
+      <c r="L20" s="6">
         <v>3.4633116995591413</v>
       </c>
-      <c r="M20" s="8">
+      <c r="M20" s="6">
         <v>47.638534727253287</v>
       </c>
-      <c r="N20" s="14">
+      <c r="N20" s="10">
         <v>79.625443005372546</v>
       </c>
-      <c r="O20" s="30">
+      <c r="O20" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="5">
+      <c r="A21" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="4">
         <v>1278101</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="4">
         <v>1278098</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>9834</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="4">
         <v>67494</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="4">
         <v>537461</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="4">
         <v>740638</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <v>2656</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="4">
         <v>12490</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="4">
         <v>459217</v>
       </c>
-      <c r="K21" s="13">
+      <c r="K21" s="9">
         <v>30</v>
       </c>
-      <c r="L21" s="8">
+      <c r="L21" s="6">
         <v>5.2808033167957769</v>
       </c>
-      <c r="M21" s="8">
+      <c r="M21" s="6">
         <v>42.051528009132298</v>
       </c>
-      <c r="N21" s="14">
+      <c r="N21" s="10">
         <v>77.981161113245349</v>
       </c>
-      <c r="O21" s="30">
+      <c r="O21" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" s="5">
+      <c r="A22" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="4">
         <v>1682332</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="4">
         <v>1839541</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="4">
         <v>5701</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="4">
         <v>152819</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="4">
         <v>304966</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="4">
         <v>1534575</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="4">
         <v>8554</v>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="4">
         <v>14255</v>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="4">
         <v>983165</v>
       </c>
-      <c r="K22" s="13">
+      <c r="K22" s="9">
         <v>30</v>
       </c>
-      <c r="L22" s="8">
+      <c r="L22" s="6">
         <v>9.0837599237249247</v>
       </c>
-      <c r="M22" s="8">
+      <c r="M22" s="6">
         <v>18.127575294293873</v>
       </c>
-      <c r="N22" s="14">
+      <c r="N22" s="10">
         <v>76.56818035916811</v>
       </c>
-      <c r="O22" s="30">
+      <c r="O22" s="13">
         <v>3733.7973859381045</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="29" t="s">
+      <c r="A23" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="4">
+        <v>80077</v>
+      </c>
+      <c r="C23" s="4">
+        <v>80077</v>
+      </c>
+      <c r="D23" s="4">
+        <v>256</v>
+      </c>
+      <c r="E23" s="4">
+        <v>409</v>
+      </c>
+      <c r="F23" s="4">
+        <v>16907</v>
+      </c>
+      <c r="G23" s="4">
+        <v>63170</v>
+      </c>
+      <c r="H23" s="4">
+        <v>284</v>
+      </c>
+      <c r="I23" s="4">
+        <v>540</v>
+      </c>
+      <c r="J23" s="4">
+        <v>42742</v>
+      </c>
+      <c r="K23" s="9">
+        <v>30</v>
+      </c>
+      <c r="L23" s="6">
+        <v>0.5107583950447695</v>
+      </c>
+      <c r="M23" s="6">
+        <v>21.11342832523696</v>
+      </c>
+      <c r="N23" s="10">
+        <v>74.489553804463213</v>
+      </c>
+      <c r="O23" s="13">
+        <v>107.74954752469391</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="5">
-        <v>80077</v>
-      </c>
-      <c r="C23" s="5">
-        <v>80077</v>
-      </c>
-      <c r="D23" s="5">
-        <v>256</v>
-      </c>
-      <c r="E23" s="5">
-        <v>409</v>
-      </c>
-      <c r="F23" s="5">
-        <v>16907</v>
-      </c>
-      <c r="G23" s="5">
-        <v>63170</v>
-      </c>
-      <c r="H23" s="5">
-        <v>284</v>
-      </c>
-      <c r="I23" s="5">
-        <v>540</v>
-      </c>
-      <c r="J23" s="5">
-        <v>42742</v>
-      </c>
-      <c r="K23" s="13">
+      <c r="B24" s="31">
+        <v>457531</v>
+      </c>
+      <c r="C24" s="31">
+        <v>457532</v>
+      </c>
+      <c r="D24" s="31">
+        <v>117</v>
+      </c>
+      <c r="E24" s="31">
+        <v>2865</v>
+      </c>
+      <c r="F24" s="31">
+        <v>9424</v>
+      </c>
+      <c r="G24" s="31">
+        <v>448108</v>
+      </c>
+      <c r="H24" s="31">
+        <v>3641</v>
+      </c>
+      <c r="I24" s="31">
+        <v>3758</v>
+      </c>
+      <c r="J24" s="31">
+        <v>285445</v>
+      </c>
+      <c r="K24" s="32">
         <v>30</v>
       </c>
-      <c r="L23" s="8">
-        <v>0.5107583950447695</v>
-      </c>
-      <c r="M23" s="8">
-        <v>21.11342832523696</v>
-      </c>
-      <c r="N23" s="14">
-        <v>74.489553804463213</v>
-      </c>
-      <c r="O23" s="30">
-        <v>107.74954752469391</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="32">
-        <v>457531</v>
-      </c>
-      <c r="C24" s="32">
-        <v>457532</v>
-      </c>
-      <c r="D24" s="32">
-        <v>117</v>
-      </c>
-      <c r="E24" s="32">
-        <v>2865</v>
-      </c>
-      <c r="F24" s="32">
-        <v>9424</v>
-      </c>
-      <c r="G24" s="32">
-        <v>448108</v>
-      </c>
-      <c r="H24" s="32">
-        <v>3641</v>
-      </c>
-      <c r="I24" s="32">
-        <v>3758</v>
-      </c>
-      <c r="J24" s="32">
-        <v>285445</v>
-      </c>
-      <c r="K24" s="33">
-        <v>30</v>
-      </c>
-      <c r="L24" s="34">
+      <c r="L24" s="33">
         <v>0.62618707803405671</v>
       </c>
-      <c r="M24" s="34">
+      <c r="M24" s="33">
         <v>2.0597511425455326</v>
       </c>
-      <c r="N24" s="35">
+      <c r="N24" s="34">
         <v>64.447873477425574</v>
       </c>
-      <c r="O24" s="36">
+      <c r="O24" s="35">
         <v>1587.0893569609509</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A18:O18"/>
-  </mergeCells>
   <conditionalFormatting sqref="L3:L17">
     <cfRule type="cellIs" dxfId="12" priority="27" operator="lessThan">
       <formula>$K$3</formula>
@@ -2182,13 +2502,77 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L19">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L19:L24">
+    <cfRule type="cellIs" dxfId="11" priority="13" operator="lessThan">
+      <formula>$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L20">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L21:L24">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L3:N17">
-    <cfRule type="cellIs" dxfId="11" priority="26" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="26" operator="greaterThan">
+      <formula>$K$4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L19:N24">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3:M6">
-    <cfRule type="cellIs" dxfId="10" priority="22" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="22" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2211,35 +2595,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M8:M17">
-    <cfRule type="cellIs" dxfId="9" priority="21" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="21" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N9">
-    <cfRule type="cellIs" dxfId="8" priority="23" operator="lessThan">
-      <formula>$K$9</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N13">
-    <cfRule type="cellIs" dxfId="7" priority="19" operator="greaterThan">
-      <formula>$K$13</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N13:N14">
-    <cfRule type="cellIs" dxfId="6" priority="20" operator="lessThan">
-      <formula>$K$9</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N14">
-    <cfRule type="cellIs" dxfId="5" priority="24" operator="equal">
-      <formula>$K$14</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="25" operator="greaterThan">
-      <formula>$K$14</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L19">
-    <cfRule type="colorScale" priority="17">
+  <conditionalFormatting sqref="M19">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
@@ -2247,7 +2608,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
@@ -2256,13 +2617,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L19:L24">
-    <cfRule type="cellIs" dxfId="3" priority="12" operator="lessThan">
+  <conditionalFormatting sqref="M19:M24">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L20">
-    <cfRule type="colorScale" priority="15">
+  <conditionalFormatting sqref="M20">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
@@ -2270,7 +2631,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
@@ -2279,8 +2640,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L21:L24">
-    <cfRule type="colorScale" priority="13">
+  <conditionalFormatting sqref="M22:M23">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
+      <formula>$K$22</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
@@ -2288,7 +2652,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="14">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
@@ -2297,13 +2661,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L19:N24">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
-      <formula>$K$4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M19">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="M24 M21">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
@@ -2311,7 +2670,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="11">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
@@ -2320,66 +2679,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M19:M24">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
-      <formula>$K$3</formula>
+  <conditionalFormatting sqref="N9">
+    <cfRule type="cellIs" dxfId="4" priority="23" operator="lessThan">
+      <formula>$K$9</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M20">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
+  <conditionalFormatting sqref="N13">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+      <formula>$K$13</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M22:M23">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
-      <formula>$K$22</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
+  <conditionalFormatting sqref="N13:N14">
+    <cfRule type="cellIs" dxfId="2" priority="20" operator="lessThan">
+      <formula>$K$9</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M24 M21">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
+  <conditionalFormatting sqref="N14">
+    <cfRule type="cellIs" dxfId="1" priority="24" operator="equal">
+      <formula>$K$14</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="25" operator="greaterThan">
+      <formula>$K$14</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add large park section: boundaries, canopy/plantable/species data, extent-box fix, species alias matching, split plantable toggle
</commit_message>
<xml_diff>
--- a/roads_data.xlsx
+++ b/roads_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed\Downloads\Aa_Canopy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7F61AD-8702-4253-81BC-EC301AFD4EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4B3947-032C-4C36-AF90-BC90993C8B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7AAB8FE-2C25-4993-9707-1AE9B1428E4B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Project area (m2)</t>
   </si>
@@ -159,6 +159,24 @@
   </si>
   <si>
     <t>Road</t>
+  </si>
+  <si>
+    <t>Large Park</t>
+  </si>
+  <si>
+    <t>Ar Rimal Park</t>
+  </si>
+  <si>
+    <t>Al Aziziyah Park</t>
+  </si>
+  <si>
+    <t>Taweeq Park</t>
+  </si>
+  <si>
+    <t>Bader Park</t>
+  </si>
+  <si>
+    <t>Al Arid Park</t>
   </si>
 </sst>
 </file>
@@ -230,7 +248,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -472,12 +490,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -540,122 +586,28 @@
     <xf numFmtId="43" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="52">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="27">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -738,36 +690,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -813,116 +735,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1396,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB4A8203-71CE-4FE6-A4FD-E83278BD534D}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:Z30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" customWidth="1"/>
@@ -2132,7 +1944,7 @@
         <v>4183.5991620404311</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="25" t="s">
         <v>29</v>
       </c>
@@ -2179,7 +1991,7 @@
         <v>5301.4341102779636</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
         <v>30</v>
       </c>
@@ -2198,7 +2010,7 @@
       <c r="N18" s="23"/>
       <c r="O18" s="23"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="28" t="s">
         <v>31</v>
       </c>
@@ -2245,7 +2057,7 @@
         <v>8329.5606031144252</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
         <v>32</v>
       </c>
@@ -2292,7 +2104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>33</v>
       </c>
@@ -2339,7 +2151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>34</v>
       </c>
@@ -2386,7 +2198,7 @@
         <v>3733.7973859381045</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>35</v>
       </c>
@@ -2433,7 +2245,7 @@
         <v>107.74954752469391</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="30" t="s">
         <v>36</v>
       </c>
@@ -2480,12 +2292,335 @@
         <v>1587.0893569609509</v>
       </c>
     </row>
+    <row r="25" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="37"/>
+      <c r="J25" s="37"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="37"/>
+      <c r="M25" s="37"/>
+      <c r="N25" s="37"/>
+      <c r="O25" s="37"/>
+      <c r="P25" s="37"/>
+      <c r="Q25" s="37"/>
+      <c r="R25" s="37"/>
+      <c r="S25" s="37"/>
+      <c r="T25" s="37"/>
+      <c r="U25" s="37"/>
+      <c r="V25" s="37"/>
+      <c r="W25" s="37"/>
+      <c r="X25" s="38"/>
+      <c r="Y25" s="39"/>
+      <c r="Z25" s="39"/>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="4">
+        <v>132158</v>
+      </c>
+      <c r="C26" s="40">
+        <v>81922</v>
+      </c>
+      <c r="D26" s="40">
+        <v>0</v>
+      </c>
+      <c r="E26" s="40">
+        <v>0</v>
+      </c>
+      <c r="F26" s="40">
+        <v>0</v>
+      </c>
+      <c r="G26" s="40">
+        <v>81922</v>
+      </c>
+      <c r="H26" s="40">
+        <v>1532</v>
+      </c>
+      <c r="I26" s="40">
+        <v>1532</v>
+      </c>
+      <c r="J26" s="40">
+        <v>43247</v>
+      </c>
+      <c r="K26" s="40">
+        <v>50</v>
+      </c>
+      <c r="L26" s="33">
+        <v>0</v>
+      </c>
+      <c r="M26" s="33">
+        <v>0</v>
+      </c>
+      <c r="N26" s="34">
+        <v>32.72370949923576</v>
+      </c>
+      <c r="O26" s="35">
+        <v>1201.4363636363637</v>
+      </c>
+      <c r="P26" s="40"/>
+      <c r="Q26" s="40"/>
+      <c r="R26" s="40"/>
+      <c r="S26" s="41"/>
+      <c r="T26" s="41"/>
+      <c r="U26" s="41"/>
+      <c r="V26" s="41"/>
+      <c r="W26" s="41"/>
+      <c r="X26" s="42"/>
+      <c r="Y26" s="39"/>
+      <c r="Z26" s="39"/>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4">
+        <v>159185</v>
+      </c>
+      <c r="C27" s="40">
+        <v>79967</v>
+      </c>
+      <c r="D27" s="40">
+        <v>48</v>
+      </c>
+      <c r="E27" s="40">
+        <v>284</v>
+      </c>
+      <c r="F27" s="40">
+        <v>1753</v>
+      </c>
+      <c r="G27" s="40">
+        <v>78214</v>
+      </c>
+      <c r="H27" s="40">
+        <v>698</v>
+      </c>
+      <c r="I27" s="40">
+        <v>746</v>
+      </c>
+      <c r="J27" s="40">
+        <v>54728</v>
+      </c>
+      <c r="K27" s="40">
+        <v>50</v>
+      </c>
+      <c r="L27" s="33">
+        <v>0.17840876967050914</v>
+      </c>
+      <c r="M27" s="33">
+        <v>1.1012344127901497</v>
+      </c>
+      <c r="N27" s="34">
+        <v>35.481358168169109</v>
+      </c>
+      <c r="O27" s="35">
+        <v>2131.3725042783799</v>
+      </c>
+      <c r="P27" s="40"/>
+      <c r="Q27" s="40"/>
+      <c r="R27" s="40"/>
+      <c r="S27" s="41"/>
+      <c r="T27" s="41"/>
+      <c r="U27" s="41"/>
+      <c r="V27" s="43"/>
+      <c r="W27" s="43"/>
+      <c r="X27" s="42"/>
+      <c r="Y27" s="39"/>
+      <c r="Z27" s="39"/>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="4">
+        <v>140509</v>
+      </c>
+      <c r="C28" s="40">
+        <v>61512</v>
+      </c>
+      <c r="D28" s="40">
+        <v>0</v>
+      </c>
+      <c r="E28" s="40">
+        <v>0</v>
+      </c>
+      <c r="F28" s="40">
+        <v>0</v>
+      </c>
+      <c r="G28" s="40">
+        <v>61512</v>
+      </c>
+      <c r="H28" s="40">
+        <v>1026</v>
+      </c>
+      <c r="I28" s="40">
+        <v>1026</v>
+      </c>
+      <c r="J28" s="40">
+        <v>28963</v>
+      </c>
+      <c r="K28" s="40">
+        <v>50</v>
+      </c>
+      <c r="L28" s="33">
+        <v>0</v>
+      </c>
+      <c r="M28" s="33">
+        <v>0</v>
+      </c>
+      <c r="N28" s="34">
+        <v>20.612914475229342</v>
+      </c>
+      <c r="O28" s="35">
+        <v>1277.3545454545454</v>
+      </c>
+      <c r="P28" s="40"/>
+      <c r="Q28" s="40"/>
+      <c r="R28" s="40"/>
+      <c r="S28" s="41"/>
+      <c r="T28" s="41"/>
+      <c r="U28" s="41"/>
+      <c r="V28" s="41"/>
+      <c r="W28" s="41"/>
+      <c r="X28" s="42"/>
+      <c r="Y28" s="39"/>
+      <c r="Z28" s="39"/>
+    </row>
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="4">
+        <v>5120</v>
+      </c>
+      <c r="C29" s="40">
+        <v>2180</v>
+      </c>
+      <c r="D29" s="40">
+        <v>19</v>
+      </c>
+      <c r="E29" s="40">
+        <v>458</v>
+      </c>
+      <c r="F29" s="40">
+        <v>926</v>
+      </c>
+      <c r="G29" s="40">
+        <v>1254</v>
+      </c>
+      <c r="H29" s="40">
+        <v>6</v>
+      </c>
+      <c r="I29" s="40">
+        <v>25</v>
+      </c>
+      <c r="J29" s="40">
+        <v>470</v>
+      </c>
+      <c r="K29" s="40">
+        <v>50</v>
+      </c>
+      <c r="L29" s="33">
+        <v>8.9453125</v>
+      </c>
+      <c r="M29" s="33">
+        <v>18.0859375</v>
+      </c>
+      <c r="N29" s="34">
+        <v>27.265625</v>
+      </c>
+      <c r="O29" s="35">
+        <v>33.52699784017279</v>
+      </c>
+      <c r="P29" s="40"/>
+      <c r="Q29" s="40"/>
+      <c r="R29" s="40"/>
+      <c r="S29" s="41"/>
+      <c r="T29" s="41"/>
+      <c r="U29" s="41"/>
+      <c r="V29" s="41"/>
+      <c r="W29" s="41"/>
+      <c r="X29" s="42"/>
+      <c r="Y29" s="39"/>
+      <c r="Z29" s="39"/>
+    </row>
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="4">
+        <v>63501</v>
+      </c>
+      <c r="C30" s="40">
+        <v>22552</v>
+      </c>
+      <c r="D30" s="40">
+        <v>4</v>
+      </c>
+      <c r="E30" s="40">
+        <v>66</v>
+      </c>
+      <c r="F30" s="40">
+        <v>179</v>
+      </c>
+      <c r="G30" s="40">
+        <v>22373</v>
+      </c>
+      <c r="H30" s="40">
+        <v>185</v>
+      </c>
+      <c r="I30" s="40">
+        <v>189</v>
+      </c>
+      <c r="J30" s="40">
+        <v>18523</v>
+      </c>
+      <c r="K30" s="40">
+        <v>50</v>
+      </c>
+      <c r="L30" s="33">
+        <v>0.10393537109651817</v>
+      </c>
+      <c r="M30" s="33">
+        <v>0.28188532464055688</v>
+      </c>
+      <c r="N30" s="34">
+        <v>29.451504700713375</v>
+      </c>
+      <c r="O30" s="35">
+        <v>705.50837988826811</v>
+      </c>
+      <c r="P30" s="40"/>
+      <c r="Q30" s="40"/>
+      <c r="R30" s="40"/>
+      <c r="S30" s="41"/>
+      <c r="T30" s="41"/>
+      <c r="U30" s="41"/>
+      <c r="V30" s="41"/>
+      <c r="W30" s="41"/>
+      <c r="X30" s="42"/>
+      <c r="Y30" s="39"/>
+      <c r="Z30" s="39"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A25:X25"/>
+  </mergeCells>
   <conditionalFormatting sqref="L3:L17">
-    <cfRule type="cellIs" dxfId="12" priority="27" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="38" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="28">
+    <cfRule type="colorScale" priority="39">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
@@ -2493,7 +2628,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="29">
+    <cfRule type="colorScale" priority="40">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
@@ -2503,6 +2638,165 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19">
+    <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L19:L24">
+    <cfRule type="cellIs" dxfId="25" priority="24" operator="lessThan">
+      <formula>$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L20">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="28">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L21:L24">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:N17">
+    <cfRule type="cellIs" dxfId="24" priority="37" operator="greaterThan">
+      <formula>$K$4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L19:N24">
+    <cfRule type="cellIs" dxfId="23" priority="15" operator="greaterThan">
+      <formula>$K$4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:M6">
+    <cfRule type="cellIs" dxfId="22" priority="33" operator="lessThan">
+      <formula>$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:M17">
+    <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M8:M17">
+    <cfRule type="cellIs" dxfId="21" priority="32" operator="lessThan">
+      <formula>$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M19">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M19:M24">
+    <cfRule type="cellIs" dxfId="20" priority="14" operator="lessThan">
+      <formula>$K$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M20">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M22:M23">
+    <cfRule type="cellIs" dxfId="19" priority="13" operator="lessThan">
+      <formula>$K$22</formula>
+    </cfRule>
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M24 M21">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
@@ -2520,13 +2814,34 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L19:L24">
-    <cfRule type="cellIs" dxfId="11" priority="13" operator="lessThan">
+  <conditionalFormatting sqref="N9">
+    <cfRule type="cellIs" dxfId="18" priority="34" operator="lessThan">
+      <formula>$K$9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N13">
+    <cfRule type="cellIs" dxfId="17" priority="12" operator="greaterThan">
+      <formula>$K$13</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N13:N14">
+    <cfRule type="cellIs" dxfId="16" priority="31" operator="lessThan">
+      <formula>$K$9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N14">
+    <cfRule type="cellIs" dxfId="15" priority="35" operator="equal">
+      <formula>$K$14</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="36" operator="greaterThan">
+      <formula>$K$14</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L26:L30">
+    <cfRule type="cellIs" dxfId="6" priority="9" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L20">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
@@ -2534,7 +2849,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
@@ -2543,125 +2858,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L21:L24">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
+  <conditionalFormatting sqref="L26:M30">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
+      <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:N17">
-    <cfRule type="cellIs" dxfId="10" priority="26" operator="greaterThan">
-      <formula>$K$4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L19:N24">
-    <cfRule type="cellIs" dxfId="9" priority="4" operator="greaterThan">
-      <formula>$K$4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M3:M6">
-    <cfRule type="cellIs" dxfId="8" priority="22" operator="lessThan">
+  <conditionalFormatting sqref="M26:M30">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M3:M17">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="31">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M8:M17">
-    <cfRule type="cellIs" dxfId="7" priority="21" operator="lessThan">
-      <formula>$K$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M19">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M19:M24">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
-      <formula>$K$3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M20">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M22:M23">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
-      <formula>$K$22</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.59999389629810485"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M24 M21">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
@@ -2679,27 +2884,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N9">
-    <cfRule type="cellIs" dxfId="4" priority="23" operator="lessThan">
-      <formula>$K$9</formula>
+  <conditionalFormatting sqref="N26:N30">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <formula>$K$26</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+      <formula>$K$26</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
+      <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N13">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
-      <formula>$K$13</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N13:N14">
-    <cfRule type="cellIs" dxfId="2" priority="20" operator="lessThan">
-      <formula>$K$9</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N14">
-    <cfRule type="cellIs" dxfId="1" priority="24" operator="equal">
-      <formula>$K$14</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="25" operator="greaterThan">
-      <formula>$K$14</formula>
+  <conditionalFormatting sqref="M29">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>$K$33</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update roads_data.xlsx with latest project figures
Wadi Umm Qassar's Current/Mature/Future KPI% recalculated automatically from the live formulas after the underlying values were updated.
</commit_message>
<xml_diff>
--- a/roads_data.xlsx
+++ b/roads_data.xlsx
@@ -1,80 +1,243 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed\Downloads\Aa_Canopy\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CFAAF5-41A1-41B8-A4FF-B1C2701F925E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>Project area (m2)</t>
+  </si>
+  <si>
+    <t>Plantable area (m2)</t>
+  </si>
+  <si>
+    <t>Current trees 
+(merged from PS and GIS)</t>
+  </si>
+  <si>
+    <t>Current canopy cover (m2)</t>
+  </si>
+  <si>
+    <t>Mature canopy cover current trees (m2) as per species</t>
+  </si>
+  <si>
+    <t>Remaining plantable Area</t>
+  </si>
+  <si>
+    <t>Potential 
+Additional 
+trees</t>
+  </si>
+  <si>
+    <t>Total trees</t>
+  </si>
+  <si>
+    <t>Potential 
+additional canopy cover (m2)</t>
+  </si>
+  <si>
+    <t>Planned 
+KPI (%)</t>
+  </si>
+  <si>
+    <t>Current KPI (%)</t>
+  </si>
+  <si>
+    <t>Current KPI mature canopy (%)</t>
+  </si>
+  <si>
+    <t>Potential Total future 
+KPI (%)</t>
+  </si>
+  <si>
+    <t>Trees to be planted to reach planned KPI</t>
+  </si>
+  <si>
+    <t>Road</t>
+  </si>
+  <si>
+    <t>Airport Road</t>
+  </si>
+  <si>
+    <t>Dammam Road</t>
+  </si>
+  <si>
+    <t>Dammam Road Riyadh Entrance</t>
+  </si>
+  <si>
+    <t>Eastern Ring Road</t>
+  </si>
+  <si>
+    <t>Jeddah Road</t>
+  </si>
+  <si>
+    <t>Khurais Road</t>
+  </si>
+  <si>
+    <t>King Fahad Road</t>
+  </si>
+  <si>
+    <t>King Khalid Road</t>
+  </si>
+  <si>
+    <t>King Salman Road</t>
+  </si>
+  <si>
+    <t>Makkah Road</t>
+  </si>
+  <si>
+    <t>Northern Ring Road</t>
+  </si>
+  <si>
+    <t>Qassim Road</t>
+  </si>
+  <si>
+    <t>Salboukh Road</t>
+  </si>
+  <si>
+    <t>Southern Ring Road</t>
+  </si>
+  <si>
+    <t>Western Ring Road</t>
+  </si>
+  <si>
+    <t>Wadi</t>
+  </si>
+  <si>
+    <t>Airport Wadi</t>
+  </si>
+  <si>
+    <t>Wadi Gudwanah</t>
+  </si>
+  <si>
+    <t>Wadi Umm Qassar</t>
+  </si>
+  <si>
+    <t>Wadi Al Laysan Linear Park</t>
+  </si>
+  <si>
+    <t>Branch of Wadi Al Laysan Phase 1 (KACST)</t>
+  </si>
+  <si>
+    <t>Branch of Wadi Al Laysan Phase 2 (KACST)</t>
+  </si>
+  <si>
+    <t>Large Park</t>
+  </si>
+  <si>
+    <t>Ar Rimal Park</t>
+  </si>
+  <si>
+    <t>Al Aziziyah Park</t>
+  </si>
+  <si>
+    <t>Taweeq Park</t>
+  </si>
+  <si>
+    <t>Bader Park</t>
+  </si>
+  <si>
+    <t>Al Arid Park</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999938962981048"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -84,14 +247,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="24">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -376,223 +533,103 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+  <cellXfs count="51">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
   </cellStyles>
-  <dxfs count="28">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="20">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -795,74 +832,14 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1182,1369 +1159,1277 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="32.42578125" customWidth="1" min="1" max="1"/>
-    <col width="26.5703125" customWidth="1" min="2" max="2"/>
-    <col width="28.5703125" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="18.7109375" customWidth="1" min="5" max="6"/>
-    <col width="17.7109375" customWidth="1" min="7" max="7"/>
-    <col width="15.7109375" customWidth="1" min="15" max="15"/>
+    <col min="1" max="1" width="32.42578125" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60.75" customHeight="1" thickBot="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="B1" s="19" t="inlineStr">
-        <is>
-          <t>Project area (m2)</t>
-        </is>
-      </c>
-      <c r="C1" s="19" t="inlineStr">
-        <is>
-          <t>Plantable area (m2)</t>
-        </is>
-      </c>
-      <c r="D1" s="20" t="inlineStr">
-        <is>
-          <t>Current trees 
-(merged from PS and GIS)</t>
-        </is>
-      </c>
-      <c r="E1" s="20" t="inlineStr">
-        <is>
-          <t>Current canopy cover (m2)</t>
-        </is>
-      </c>
-      <c r="F1" s="20" t="inlineStr">
-        <is>
-          <t>Mature canopy cover current trees (m2) as per species</t>
-        </is>
-      </c>
-      <c r="G1" s="20" t="inlineStr">
-        <is>
-          <t>Remaining plantable Area</t>
-        </is>
-      </c>
-      <c r="H1" s="20" t="inlineStr">
-        <is>
-          <t>Potential 
-Additional 
-trees</t>
-        </is>
-      </c>
-      <c r="I1" s="19" t="inlineStr">
-        <is>
-          <t>Total trees</t>
-        </is>
-      </c>
-      <c r="J1" s="20" t="inlineStr">
-        <is>
-          <t>Potential 
-additional canopy cover (m2)</t>
-        </is>
-      </c>
-      <c r="K1" s="20" t="inlineStr">
-        <is>
-          <t>Planned 
-KPI (%)</t>
-        </is>
-      </c>
-      <c r="L1" s="20" t="inlineStr">
-        <is>
-          <t>Current KPI (%)</t>
-        </is>
-      </c>
-      <c r="M1" s="20" t="inlineStr">
-        <is>
-          <t>Current KPI mature canopy (%)</t>
-        </is>
-      </c>
-      <c r="N1" s="20" t="inlineStr">
-        <is>
-          <t>Potential Total future 
-KPI (%)</t>
-        </is>
-      </c>
-      <c r="O1" s="21" t="inlineStr">
-        <is>
-          <t>Trees to be planted to reach planned KPI</t>
-        </is>
+    <row r="1" spans="1:15" ht="60.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Road</t>
-        </is>
-      </c>
-      <c r="B2" s="23" t="n"/>
-      <c r="C2" s="23" t="n"/>
-      <c r="D2" s="23" t="n"/>
-      <c r="E2" s="23" t="n"/>
-      <c r="F2" s="23" t="n"/>
-      <c r="G2" s="23" t="n"/>
-      <c r="H2" s="23" t="n"/>
-      <c r="I2" s="23" t="n"/>
-      <c r="J2" s="23" t="n"/>
-      <c r="K2" s="23" t="n"/>
-      <c r="L2" s="23" t="n"/>
-      <c r="M2" s="23" t="n"/>
-      <c r="N2" s="23" t="n"/>
-      <c r="O2" s="23" t="n"/>
+    <row r="2" spans="1:15" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Airport Road</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3">
         <v>5339843</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="3">
         <v>3105072</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="3">
         <v>19360</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="3">
         <v>288353</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="3">
         <v>1086200</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="3">
         <v>2018871</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="3">
         <v>10853</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="3">
         <v>30243</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="J3" s="3">
         <v>1396924</v>
       </c>
-      <c r="K3" s="7" t="n">
+      <c r="K3" s="7">
         <v>12</v>
       </c>
       <c r="L3" s="5">
-        <f>100/B3*E3</f>
+        <f t="shared" ref="L3:L17" si="0">100/B3*E3</f>
         <v>5.4000276787163966</v>
       </c>
       <c r="M3" s="5">
-        <f>100/B3*F3</f>
+        <f t="shared" ref="M3:M17" si="1">100/B3*F3</f>
         <v>20.34142202308195</v>
       </c>
       <c r="N3" s="8">
-        <f>100/B3*(F3+J3)</f>
-        <v>46.50181662644388</v>
-      </c>
-      <c r="O3" s="24" t="n">
+        <f t="shared" ref="N3:N17" si="2">100/B3*(F3+J3)</f>
+        <v>46.501816626443883</v>
+      </c>
+      <c r="O3" s="24">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Dammam Road</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="4">
         <v>3503507</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="3">
         <v>2196951</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="3">
         <v>7508</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="3">
         <v>3203</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="3">
         <v>588536</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="3">
         <v>1608415</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="3">
         <v>11308</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="3">
         <v>18816</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="3">
         <v>1124890</v>
       </c>
-      <c r="K4" s="9" t="n">
+      <c r="K4" s="9">
         <v>12</v>
       </c>
       <c r="L4" s="6">
-        <f>100/B4*E4</f>
-        <v>0.0914226801887366</v>
+        <f t="shared" si="0"/>
+        <v>9.1422680188736602E-2</v>
       </c>
       <c r="M4" s="6">
-        <f>100/B4*F4</f>
+        <f t="shared" si="1"/>
         <v>16.79848220654333</v>
       </c>
       <c r="N4" s="10">
-        <f>100/B4*(F4+J4)</f>
-        <v>48.90602473464446</v>
-      </c>
-      <c r="O4" s="13" t="n">
+        <f t="shared" si="2"/>
+        <v>48.906024734644461</v>
+      </c>
+      <c r="O4" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Dammam Road Riyadh Entrance</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="4">
         <v>1858085</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="3">
         <v>799865</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="3">
         <v>3168</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="3">
         <v>12986</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="3">
         <v>197600</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="3">
         <v>602265</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="3">
         <v>3875</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="3">
         <v>7043</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="J5" s="3">
         <v>414882</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K5" s="11">
         <v>12</v>
       </c>
       <c r="L5" s="6">
-        <f>100/B5*E5</f>
-        <v>0.6988916007609985</v>
+        <f t="shared" si="0"/>
+        <v>0.69889160076099854</v>
       </c>
       <c r="M5" s="6">
-        <f>100/B5*F5</f>
+        <f t="shared" si="1"/>
         <v>10.634604983087426</v>
       </c>
       <c r="N5" s="10">
-        <f>100/B5*(F5+J5)</f>
-        <v>32.96307757718296</v>
-      </c>
-      <c r="O5" s="13" t="n">
-        <v>406.7449068825911</v>
+        <f t="shared" si="2"/>
+        <v>32.963077577182958</v>
+      </c>
+      <c r="O5" s="13">
+        <v>406.74490688259112</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Eastern Ring Road</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="4">
         <v>3612799</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="3">
         <v>1285169</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="3">
         <v>10558</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="3">
         <v>107102</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="3">
         <v>467496</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="3">
         <v>817673</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="3">
         <v>5160</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="3">
         <v>15718</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J6" s="3">
         <v>522325</v>
       </c>
-      <c r="K6" s="11" t="n">
+      <c r="K6" s="11">
         <v>12</v>
       </c>
       <c r="L6" s="6">
-        <f>100/B6*E6</f>
+        <f t="shared" si="0"/>
         <v>2.964515878132163</v>
       </c>
       <c r="M6" s="6">
-        <f>100/B6*F6</f>
+        <f t="shared" si="1"/>
         <v>12.939994724312092</v>
       </c>
       <c r="N6" s="10">
-        <f>100/B6*(F6+J6)</f>
+        <f t="shared" si="2"/>
         <v>27.397621622459486</v>
       </c>
-      <c r="O6" s="13" t="n">
+      <c r="O6" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Jeddah Road</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4">
         <v>450056</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="3">
         <v>144911</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="3">
         <v>1516</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="3">
         <v>14702</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="3">
         <v>82945</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G7" s="3">
         <v>61966</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="3">
         <v>363</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I7" s="3">
         <v>1879</v>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="J7" s="3">
         <v>50040</v>
       </c>
-      <c r="K7" s="11" t="n">
+      <c r="K7" s="11">
         <v>12</v>
       </c>
       <c r="L7" s="6">
-        <f>100/B7*E7</f>
-        <v>3.266704587873509</v>
+        <f t="shared" si="0"/>
+        <v>3.2667045878735088</v>
       </c>
       <c r="M7" s="6">
-        <f>100/B7*F7</f>
-        <v>18.42992871998151</v>
+        <f t="shared" si="1"/>
+        <v>18.429928719981511</v>
       </c>
       <c r="N7" s="10">
-        <f>100/B7*(F7+J7)</f>
-        <v>29.54854506994685</v>
-      </c>
-      <c r="O7" s="13" t="n">
+        <f t="shared" si="2"/>
+        <v>29.548545069946851</v>
+      </c>
+      <c r="O7" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Khurais Road</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4">
         <v>2322528</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="3">
         <v>739346</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="3">
         <v>1059</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="3">
         <v>1371</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="3">
         <v>62539</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="3">
         <v>676807</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="3">
         <v>4893</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="3">
         <v>5952</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="J8" s="3">
         <v>499072</v>
       </c>
-      <c r="K8" s="11" t="n">
+      <c r="K8" s="11">
         <v>12</v>
       </c>
       <c r="L8" s="6">
-        <f>100/B8*E8</f>
-        <v>0.059030504691439674</v>
+        <f t="shared" si="0"/>
+        <v>5.9030504691439674E-2</v>
       </c>
       <c r="M8" s="6">
-        <f>100/B8*F8</f>
+        <f t="shared" si="1"/>
         <v>2.6927124237038265</v>
       </c>
       <c r="N8" s="10">
-        <f>100/B8*(F8+J8)</f>
-        <v>24.18102171426997</v>
-      </c>
-      <c r="O8" s="13" t="n">
-        <v>3660.404823230304</v>
+        <f t="shared" si="2"/>
+        <v>24.181021714269971</v>
+      </c>
+      <c r="O8" s="13">
+        <v>3660.4048232303039</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>King Fahad Road</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="4">
         <v>567004</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="3">
         <v>63865</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="3">
         <v>583</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="3">
         <v>8174</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="3">
         <v>21608</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" s="3">
         <v>42257</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="3">
         <v>325</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I9" s="3">
         <v>908</v>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="J9" s="3">
         <v>28499</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="K9" s="11">
         <v>15</v>
       </c>
       <c r="L9" s="6">
-        <f>100/B9*E9</f>
+        <f t="shared" si="0"/>
         <v>1.4416124048507595</v>
       </c>
       <c r="M9" s="6">
-        <f>100/B9*F9</f>
+        <f t="shared" si="1"/>
         <v>3.8109078595565467</v>
       </c>
       <c r="N9" s="10">
-        <f>100/B9*(F9+J9)</f>
-        <v>8.837151060662713</v>
-      </c>
-      <c r="O9" s="13" t="n">
+        <f t="shared" si="2"/>
+        <v>8.8371510606627126</v>
+      </c>
+      <c r="O9" s="13">
         <v>1711.728794890781</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>King Khalid Road</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="4">
         <v>2098017</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="3">
         <v>725672</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="3">
         <v>5806</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="3">
         <v>95034</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="3">
         <v>309776</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="3">
         <v>415896</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="3">
         <v>2252</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" s="3">
         <v>8058</v>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="J10" s="3">
         <v>267634</v>
       </c>
-      <c r="K10" s="11" t="n">
+      <c r="K10" s="11">
         <v>15</v>
       </c>
       <c r="L10" s="6">
-        <f>100/B10*E10</f>
+        <f t="shared" si="0"/>
         <v>4.5297059080074185</v>
       </c>
       <c r="M10" s="6">
-        <f>100/B10*F10</f>
+        <f t="shared" si="1"/>
         <v>14.76518064438944</v>
       </c>
       <c r="N10" s="10">
-        <f>100/B10*(F10+J10)</f>
+        <f t="shared" si="2"/>
         <v>27.521702636346607</v>
       </c>
-      <c r="O10" s="13" t="n">
-        <v>92.33623424668136</v>
+      <c r="O10" s="13">
+        <v>92.336234246681357</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>King Salman Road</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="4">
         <v>1664978</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="3">
         <v>584392</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="3">
         <v>4005</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="3">
         <v>38978</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="3">
         <v>197462</v>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="G11" s="3">
         <v>386930</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="3">
         <v>2056</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="I11" s="3">
         <v>6061</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="J11" s="3">
         <v>317712</v>
       </c>
-      <c r="K11" s="11" t="n">
+      <c r="K11" s="11">
         <v>15</v>
       </c>
       <c r="L11" s="6">
-        <f>100/B11*E11</f>
-        <v>2.34105195383963</v>
+        <f t="shared" si="0"/>
+        <v>2.3410519538396302</v>
       </c>
       <c r="M11" s="6">
-        <f>100/B11*F11</f>
+        <f t="shared" si="1"/>
         <v>11.859736284803763</v>
       </c>
       <c r="N11" s="10">
-        <f>100/B11*(F11+J11)</f>
-        <v>30.94179022185278</v>
-      </c>
-      <c r="O11" s="13" t="n">
-        <v>1060.458333755356</v>
+        <f t="shared" si="2"/>
+        <v>30.941790221852781</v>
+      </c>
+      <c r="O11" s="13">
+        <v>1060.4583337553561</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Makkah Road</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="4">
         <v>1495231</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="3">
         <v>314326</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="3">
         <v>2288</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="3">
         <v>33528</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="3">
         <v>105263</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G12" s="3">
         <v>209063</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="3">
         <v>1581</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="I12" s="3">
         <v>3869</v>
       </c>
-      <c r="J12" s="3" t="n">
+      <c r="J12" s="3">
         <v>168335</v>
       </c>
-      <c r="K12" s="11" t="n">
+      <c r="K12" s="11">
         <v>15</v>
       </c>
       <c r="L12" s="6">
-        <f>100/B12*E12</f>
-        <v>2.242329111689097</v>
+        <f t="shared" si="0"/>
+        <v>2.2423291116890969</v>
       </c>
       <c r="M12" s="6">
-        <f>100/B12*F12</f>
+        <f t="shared" si="1"/>
         <v>7.039915571573891</v>
       </c>
       <c r="N12" s="10">
-        <f>100/B12*(F12+J12)</f>
+        <f t="shared" si="2"/>
         <v>18.298042242302362</v>
       </c>
-      <c r="O12" s="13" t="n">
-        <v>2587.058464987697</v>
+      <c r="O12" s="13">
+        <v>2587.0584649876969</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Northern Ring Road</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4">
         <v>1168715</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="3">
         <v>196100</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="3">
         <v>3110</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="3">
         <v>29624</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="3">
         <v>126697</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="G13" s="3">
         <v>69403</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H13" s="3">
         <v>497</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" s="3">
         <v>3607</v>
       </c>
-      <c r="J13" s="3" t="n">
+      <c r="J13" s="3">
         <v>45784</v>
       </c>
-      <c r="K13" s="11" t="n">
+      <c r="K13" s="11">
         <v>12</v>
       </c>
       <c r="L13" s="6">
-        <f>100/B13*E13</f>
+        <f t="shared" si="0"/>
         <v>2.5347497037344433</v>
       </c>
       <c r="M13" s="6">
-        <f>100/B13*F13</f>
+        <f t="shared" si="1"/>
         <v>10.840709668310923</v>
       </c>
       <c r="N13" s="10">
-        <f>100/B13*(F13+J13)</f>
+        <f t="shared" si="2"/>
         <v>14.75817457635095</v>
       </c>
-      <c r="O13" s="13" t="n">
-        <v>332.579050806254</v>
+      <c r="O13" s="13">
+        <v>332.57905080625397</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Qassim Road</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="4">
         <v>290518</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="3">
         <v>39999</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="3">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="3">
         <v>0</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="3">
         <v>0</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G14" s="3">
         <v>39999</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="3">
         <v>732</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="I14" s="3">
         <v>732</v>
       </c>
-      <c r="J14" s="3" t="n">
+      <c r="J14" s="3">
         <v>20664</v>
       </c>
-      <c r="K14" s="11" t="n">
+      <c r="K14" s="11">
         <v>12</v>
       </c>
       <c r="L14" s="6">
-        <f>100/B14*E14</f>
-        <v>0.0</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="M14" s="6">
-        <f>100/B14*F14</f>
-        <v>0.0</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="N14" s="10">
-        <f>100/B14*(F14+J14)</f>
-        <v>7.11281228701836</v>
-      </c>
-      <c r="O14" s="13" t="n">
-        <v>633.8574545454545</v>
+        <f t="shared" si="2"/>
+        <v>7.1128122870183601</v>
+      </c>
+      <c r="O14" s="13">
+        <v>633.85745454545452</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Salboukh Road</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="4">
         <v>2409239</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="3">
         <v>1166044</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="3">
         <v>1360</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="3">
         <v>4689</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="3">
         <v>117471</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G15" s="3">
         <v>1048573</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H15" s="3">
         <v>8430</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I15" s="3">
         <v>9790</v>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="J15" s="3">
         <v>652419</v>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="K15" s="11">
         <v>12</v>
       </c>
       <c r="L15" s="6">
-        <f>100/B15*E15</f>
+        <f t="shared" si="0"/>
         <v>0.19462577187236302</v>
       </c>
       <c r="M15" s="6">
-        <f>100/B15*F15</f>
-        <v>4.875854989895149</v>
+        <f t="shared" si="1"/>
+        <v>4.8758549898951493</v>
       </c>
       <c r="N15" s="10">
-        <f>100/B15*(F15+J15)</f>
+        <f t="shared" si="2"/>
         <v>31.955733739990094</v>
       </c>
-      <c r="O15" s="13" t="n">
-        <v>1987.105283857292</v>
+      <c r="O15" s="13">
+        <v>1987.1052838572921</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Southern Ring Road</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="4">
         <v>3469847</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="3">
         <v>1184771</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="3">
         <v>2940</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="3">
         <v>77622</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="3">
         <v>171846</v>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="G16" s="3">
         <v>1012926</v>
       </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="3">
         <v>8307</v>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="I16" s="3">
         <v>11247</v>
       </c>
-      <c r="J16" s="3" t="n">
+      <c r="J16" s="3">
         <v>650917</v>
       </c>
-      <c r="K16" s="11" t="n">
+      <c r="K16" s="11">
         <v>12</v>
       </c>
       <c r="L16" s="6">
-        <f>100/B16*E16</f>
+        <f t="shared" si="0"/>
         <v>2.2370438811855395</v>
       </c>
       <c r="M16" s="6">
-        <f>100/B16*F16</f>
-        <v>4.952552662984853</v>
+        <f t="shared" si="1"/>
+        <v>4.9525526629848526</v>
       </c>
       <c r="N16" s="10">
-        <f>100/B16*(F16+J16)</f>
+        <f t="shared" si="2"/>
         <v>23.711794785187937</v>
       </c>
-      <c r="O16" s="13" t="n">
-        <v>4183.599162040431</v>
+      <c r="O16" s="13">
+        <v>4183.5991620404311</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>Western Ring Road</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="n">
+    <row r="17" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="14">
         <v>2610463</v>
       </c>
-      <c r="C17" s="26" t="n">
+      <c r="C17" s="26">
         <v>900928</v>
       </c>
-      <c r="D17" s="26" t="n">
+      <c r="D17" s="26">
         <v>1131</v>
       </c>
-      <c r="E17" s="26" t="n">
+      <c r="E17" s="26">
         <v>28105</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="26">
         <v>55079</v>
       </c>
-      <c r="G17" s="26" t="n">
+      <c r="G17" s="26">
         <v>845849</v>
       </c>
-      <c r="H17" s="26" t="n">
+      <c r="H17" s="26">
         <v>7197</v>
       </c>
-      <c r="I17" s="26" t="n">
+      <c r="I17" s="26">
         <v>8328</v>
       </c>
-      <c r="J17" s="26" t="n">
+      <c r="J17" s="26">
         <v>564240</v>
       </c>
-      <c r="K17" s="27" t="n">
+      <c r="K17" s="27">
         <v>12</v>
       </c>
       <c r="L17" s="15">
-        <f>100/B17*E17</f>
+        <f t="shared" si="0"/>
         <v>1.0766289351735687</v>
       </c>
       <c r="M17" s="15">
-        <f>100/B17*F17</f>
+        <f t="shared" si="1"/>
         <v>2.1099322227512896</v>
       </c>
       <c r="N17" s="16">
-        <f>100/B17*(F17+J17)</f>
+        <f t="shared" si="2"/>
         <v>23.724488720966356</v>
       </c>
-      <c r="O17" s="17" t="n">
-        <v>5301.434110277964</v>
+      <c r="O17" s="17">
+        <v>5301.4341102779636</v>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A18" s="22" t="inlineStr">
-        <is>
-          <t>Wadi</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="23" t="n"/>
-      <c r="D18" s="23" t="n"/>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="23" t="n"/>
-      <c r="G18" s="23" t="n"/>
-      <c r="H18" s="23" t="n"/>
-      <c r="I18" s="23" t="n"/>
-      <c r="J18" s="23" t="n"/>
-      <c r="K18" s="23" t="n"/>
-      <c r="L18" s="23" t="n"/>
-      <c r="M18" s="23" t="n"/>
-      <c r="N18" s="23" t="n"/>
-      <c r="O18" s="23" t="n"/>
+    <row r="18" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
     </row>
-    <row r="19">
-      <c r="A19" s="28" t="inlineStr">
-        <is>
-          <t>Airport Wadi</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="n">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A19" s="28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="29">
         <v>9298927</v>
       </c>
-      <c r="C19" s="29" t="n">
+      <c r="C19" s="29">
         <v>8673006</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="29">
         <v>679</v>
       </c>
-      <c r="E19" s="29" t="n">
+      <c r="E19" s="29">
         <v>6296</v>
       </c>
-      <c r="F19" s="29" t="n">
+      <c r="F19" s="29">
         <v>49062</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="29">
         <v>8623944</v>
       </c>
-      <c r="H19" s="29" t="n">
+      <c r="H19" s="29">
         <v>58495</v>
       </c>
-      <c r="I19" s="29" t="n">
+      <c r="I19" s="29">
         <v>59174</v>
       </c>
-      <c r="J19" s="29" t="n">
+      <c r="J19" s="29">
         <v>4666380</v>
       </c>
-      <c r="K19" s="7" t="n">
+      <c r="K19" s="7">
         <v>7</v>
       </c>
       <c r="L19" s="5">
-        <f>100/B19*E19</f>
-        <v>0.06770673648690864</v>
+        <f t="shared" ref="L19:L24" si="3">100/B19*E19</f>
+        <v>6.7706736486908642E-2</v>
       </c>
       <c r="M19" s="5">
-        <f>100/B19*F19</f>
-        <v>0.5276092607243825</v>
+        <f t="shared" ref="M19:M24" si="4">100/B19*F19</f>
+        <v>0.52760926072438252</v>
       </c>
       <c r="N19" s="8">
-        <f>100/B19*(F19+J19)</f>
-        <v>50.70952809931726</v>
-      </c>
-      <c r="O19" s="24" t="n">
-        <v>8329.560603114425</v>
+        <f t="shared" ref="N19:N24" si="5">100/B19*(F19+J19)</f>
+        <v>50.709528099317261</v>
+      </c>
+      <c r="O19" s="24">
+        <v>8329.5606031144252</v>
       </c>
     </row>
-    <row r="20" customFormat="1" s="57">
-      <c r="A20" s="51" t="inlineStr">
-        <is>
-          <t>Wadi Gudwanah</t>
-        </is>
-      </c>
-      <c r="B20" s="52" t="n">
+    <row r="20" spans="1:26" s="47" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="41">
         <v>663931</v>
       </c>
-      <c r="C20" s="52" t="n">
+      <c r="C20" s="41">
         <v>379631</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" s="47">
         <v>7566</v>
       </c>
-      <c r="E20" s="52" t="n">
+      <c r="E20" s="41">
         <v>13354</v>
       </c>
-      <c r="F20" s="52" t="n">
+      <c r="F20" s="41">
         <v>39071</v>
       </c>
-      <c r="G20" s="52" t="n">
+      <c r="G20" s="41">
         <v>350019</v>
       </c>
-      <c r="H20" s="52" t="n">
+      <c r="H20" s="41">
         <v>3541</v>
       </c>
-      <c r="I20" s="52" t="n">
+      <c r="I20" s="41">
         <v>11107</v>
       </c>
-      <c r="J20" s="52" t="n">
+      <c r="J20" s="41">
         <v>27343</v>
       </c>
-      <c r="K20" s="53" t="n">
+      <c r="K20" s="43">
         <v>30</v>
       </c>
-      <c r="L20" s="54">
-        <f>100/B20*E20</f>
+      <c r="L20" s="44">
+        <f t="shared" si="3"/>
         <v>2.011353589454326</v>
       </c>
-      <c r="M20" s="54">
-        <f>100/B20*F20</f>
-        <v>5.884798269699713</v>
-      </c>
-      <c r="N20" s="55">
-        <f>100/B20*(F20+J20)</f>
+      <c r="M20" s="44">
+        <f t="shared" si="4"/>
+        <v>5.8847982696997132</v>
+      </c>
+      <c r="N20" s="45">
+        <f t="shared" si="5"/>
         <v>10.003147917479378</v>
       </c>
-      <c r="O20" s="56" t="n">
+      <c r="O20" s="46">
         <v>4354</v>
       </c>
     </row>
-    <row r="21" customFormat="1" s="47">
-      <c r="A21" s="42" t="inlineStr">
-        <is>
-          <t>Wadi Umm Qassar</t>
-        </is>
-      </c>
-      <c r="B21" s="41" t="n">
+    <row r="21" spans="1:26" s="47" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="41">
         <v>1278101</v>
       </c>
-      <c r="C21" s="41" t="n">
-        <v>347135</v>
-      </c>
-      <c r="D21" t="n">
+      <c r="C21" s="41">
+        <v>462167</v>
+      </c>
+      <c r="D21" s="47">
         <v>10714</v>
       </c>
-      <c r="E21" s="41" t="n">
-        <v>42729</v>
-      </c>
-      <c r="F21" s="41" t="n">
-        <v>46053</v>
-      </c>
-      <c r="G21" s="41" t="n">
-        <v>331708</v>
-      </c>
-      <c r="H21" s="41" t="n">
-        <v>3817</v>
-      </c>
-      <c r="I21" s="41" t="n">
-        <v>14531</v>
-      </c>
-      <c r="J21" s="41" t="n">
-        <v>27029</v>
-      </c>
-      <c r="K21" s="43" t="n">
+      <c r="E21" s="41">
+        <v>21533</v>
+      </c>
+      <c r="F21" s="41">
+        <v>46054</v>
+      </c>
+      <c r="G21" s="41">
+        <v>434268</v>
+      </c>
+      <c r="H21" s="41">
+        <v>4510</v>
+      </c>
+      <c r="I21" s="41">
+        <v>15224</v>
+      </c>
+      <c r="J21" s="41">
+        <v>32415</v>
+      </c>
+      <c r="K21" s="43">
         <v>30</v>
       </c>
       <c r="L21" s="44">
-        <f>100/B21*E21</f>
-        <v>3.3431630207628347</v>
+        <f t="shared" si="3"/>
+        <v>1.6847651320200827</v>
       </c>
       <c r="M21" s="44">
-        <f>100/B21*F21</f>
-        <v>3.603236363949328</v>
+        <f t="shared" si="4"/>
+        <v>3.6033146050273022</v>
       </c>
       <c r="N21" s="45">
-        <f>100/B21*(F21+J21)</f>
-        <v>5.718014460516031</v>
-      </c>
-      <c r="O21" s="46" t="n">
+        <f t="shared" si="5"/>
+        <v>6.1394991475634546</v>
+      </c>
+      <c r="O21" s="46">
         <v>6078</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Wadi Al Laysan Linear Park</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="4">
         <v>1682332</v>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="4">
         <v>1839541</v>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="D22" s="4">
         <v>5701</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="4">
         <v>152819</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="F22" s="4">
         <v>304966</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="G22" s="4">
         <v>1534575</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="H22" s="4">
         <v>8554</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="I22" s="4">
         <v>14255</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="J22" s="4">
         <v>983165</v>
       </c>
-      <c r="K22" s="9" t="n">
+      <c r="K22" s="9">
         <v>30</v>
       </c>
       <c r="L22" s="6">
-        <f>100/B22*E22</f>
-        <v>9.083759923724925</v>
+        <f t="shared" si="3"/>
+        <v>9.0837599237249247</v>
       </c>
       <c r="M22" s="6">
-        <f>100/B22*F22</f>
+        <f t="shared" si="4"/>
         <v>18.127575294293873</v>
       </c>
       <c r="N22" s="10">
-        <f>100/B22*(F22+J22)</f>
+        <f t="shared" si="5"/>
         <v>76.56818035916811</v>
       </c>
-      <c r="O22" s="13" t="n">
+      <c r="O22" s="13">
         <v>3733.797385938105</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Branch of Wadi Al Laysan Phase 1 (KACST)</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="4">
         <v>80077</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="4">
         <v>80077</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="4">
         <v>256</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="4">
         <v>409</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F23" s="4">
         <v>16907</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="G23" s="4">
         <v>63170</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="H23" s="4">
         <v>284</v>
       </c>
-      <c r="I23" s="4" t="n">
+      <c r="I23" s="4">
         <v>540</v>
       </c>
-      <c r="J23" s="4" t="n">
+      <c r="J23" s="4">
         <v>42742</v>
       </c>
-      <c r="K23" s="9" t="n">
+      <c r="K23" s="9">
         <v>30</v>
       </c>
       <c r="L23" s="6">
-        <f>100/B23*E23</f>
+        <f t="shared" si="3"/>
         <v>0.5107583950447695</v>
       </c>
       <c r="M23" s="6">
-        <f>100/B23*F23</f>
+        <f t="shared" si="4"/>
         <v>21.11342832523696</v>
       </c>
       <c r="N23" s="10">
-        <f>100/B23*(F23+J23)</f>
-        <v>74.48955380446321</v>
-      </c>
-      <c r="O23" s="13" t="n">
+        <f t="shared" si="5"/>
+        <v>74.489553804463213</v>
+      </c>
+      <c r="O23" s="13">
         <v>107.7495475246939</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Branch of Wadi Al Laysan Phase 2 (KACST)</t>
-        </is>
-      </c>
-      <c r="B24" s="31" t="n">
+    <row r="24" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="31">
         <v>457531</v>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="31">
         <v>457532</v>
       </c>
-      <c r="D24" s="31" t="n">
+      <c r="D24" s="31">
         <v>117</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="31">
         <v>2865</v>
       </c>
-      <c r="F24" s="31" t="n">
+      <c r="F24" s="31">
         <v>9424</v>
       </c>
-      <c r="G24" s="31" t="n">
+      <c r="G24" s="31">
         <v>448108</v>
       </c>
-      <c r="H24" s="31" t="n">
+      <c r="H24" s="31">
         <v>3641</v>
       </c>
-      <c r="I24" s="31" t="n">
+      <c r="I24" s="31">
         <v>3758</v>
       </c>
-      <c r="J24" s="31" t="n">
+      <c r="J24" s="31">
         <v>285445</v>
       </c>
-      <c r="K24" s="32" t="n">
+      <c r="K24" s="32">
         <v>30</v>
       </c>
       <c r="L24" s="33">
-        <f>100/B24*E24</f>
-        <v>0.6261870780340567</v>
+        <f t="shared" si="3"/>
+        <v>0.62618707803405671</v>
       </c>
       <c r="M24" s="33">
-        <f>100/B24*F24</f>
+        <f t="shared" si="4"/>
         <v>2.0597511425455326</v>
       </c>
       <c r="N24" s="34">
-        <f>100/B24*(F24+J24)</f>
-        <v>64.44787347742557</v>
-      </c>
-      <c r="O24" s="35" t="n">
-        <v>1587.089356960951</v>
+        <f t="shared" si="5"/>
+        <v>64.447873477425574</v>
+      </c>
+      <c r="O24" s="35">
+        <v>1587.0893569609509</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A25" s="58" t="inlineStr">
-        <is>
-          <t>Large Park</t>
-        </is>
-      </c>
-      <c r="B25" s="59" t="n"/>
-      <c r="C25" s="59" t="n"/>
-      <c r="D25" s="59" t="n"/>
-      <c r="E25" s="59" t="n"/>
-      <c r="F25" s="59" t="n"/>
-      <c r="G25" s="59" t="n"/>
-      <c r="H25" s="59" t="n"/>
-      <c r="I25" s="59" t="n"/>
-      <c r="J25" s="59" t="n"/>
-      <c r="K25" s="59" t="n"/>
-      <c r="L25" s="59" t="n"/>
-      <c r="M25" s="59" t="n"/>
-      <c r="N25" s="59" t="n"/>
-      <c r="O25" s="59" t="n"/>
-      <c r="P25" s="59" t="n"/>
-      <c r="Q25" s="59" t="n"/>
-      <c r="R25" s="59" t="n"/>
-      <c r="S25" s="59" t="n"/>
-      <c r="T25" s="59" t="n"/>
-      <c r="U25" s="59" t="n"/>
-      <c r="V25" s="59" t="n"/>
-      <c r="W25" s="59" t="n"/>
-      <c r="X25" s="60" t="n"/>
-      <c r="Y25" s="36" t="n"/>
-      <c r="Z25" s="36" t="n"/>
+    <row r="25" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="49"/>
+      <c r="K25" s="49"/>
+      <c r="L25" s="49"/>
+      <c r="M25" s="49"/>
+      <c r="N25" s="49"/>
+      <c r="O25" s="49"/>
+      <c r="P25" s="49"/>
+      <c r="Q25" s="49"/>
+      <c r="R25" s="49"/>
+      <c r="S25" s="49"/>
+      <c r="T25" s="49"/>
+      <c r="U25" s="49"/>
+      <c r="V25" s="49"/>
+      <c r="W25" s="49"/>
+      <c r="X25" s="50"/>
+      <c r="Y25" s="36"/>
+      <c r="Z25" s="36"/>
     </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Ar Rimal Park</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="4">
         <v>132158</v>
       </c>
-      <c r="C26" s="37" t="n">
+      <c r="C26" s="37">
         <v>81922</v>
       </c>
-      <c r="D26" s="37" t="n">
+      <c r="D26" s="37">
         <v>0</v>
       </c>
-      <c r="E26" s="37" t="n">
+      <c r="E26" s="37">
         <v>0</v>
       </c>
-      <c r="F26" s="37" t="n">
+      <c r="F26" s="37">
         <v>0</v>
       </c>
-      <c r="G26" s="37" t="n">
+      <c r="G26" s="37">
         <v>81922</v>
       </c>
-      <c r="H26" s="37" t="n">
+      <c r="H26" s="37">
         <v>1532</v>
       </c>
-      <c r="I26" s="37" t="n">
+      <c r="I26" s="37">
         <v>1532</v>
       </c>
-      <c r="J26" s="37" t="n">
+      <c r="J26" s="37">
         <v>43247</v>
       </c>
-      <c r="K26" s="37" t="n">
+      <c r="K26" s="37">
         <v>50</v>
       </c>
       <c r="L26" s="33">
         <f>100/B26*E26</f>
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M26" s="33">
         <f>100/B26*F26</f>
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N26" s="34">
         <f>100/B26*(F26+J26)</f>
         <v>32.72370949923576</v>
       </c>
-      <c r="O26" s="35" t="n">
-        <v>1201.436363636364</v>
-      </c>
-      <c r="P26" s="37" t="n"/>
-      <c r="Q26" s="37" t="n"/>
-      <c r="R26" s="37" t="n"/>
-      <c r="S26" s="38" t="n"/>
-      <c r="T26" s="38" t="n"/>
-      <c r="U26" s="38" t="n"/>
-      <c r="V26" s="38" t="n"/>
-      <c r="W26" s="38" t="n"/>
-      <c r="X26" s="39" t="n"/>
-      <c r="Y26" s="36" t="n"/>
-      <c r="Z26" s="36" t="n"/>
+      <c r="O26" s="35">
+        <v>1201.4363636363639</v>
+      </c>
+      <c r="P26" s="37"/>
+      <c r="Q26" s="37"/>
+      <c r="R26" s="37"/>
+      <c r="S26" s="38"/>
+      <c r="T26" s="38"/>
+      <c r="U26" s="38"/>
+      <c r="V26" s="38"/>
+      <c r="W26" s="38"/>
+      <c r="X26" s="39"/>
+      <c r="Y26" s="36"/>
+      <c r="Z26" s="36"/>
     </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Al Aziziyah Park</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="4">
         <v>159185</v>
       </c>
-      <c r="C27" s="37" t="n">
+      <c r="C27" s="37">
         <v>79967</v>
       </c>
-      <c r="D27" s="37" t="n">
+      <c r="D27" s="37">
         <v>48</v>
       </c>
-      <c r="E27" s="37" t="n">
+      <c r="E27" s="37">
         <v>284</v>
       </c>
-      <c r="F27" s="37" t="n">
+      <c r="F27" s="37">
         <v>1753</v>
       </c>
-      <c r="G27" s="37" t="n">
+      <c r="G27" s="37">
         <v>78214</v>
       </c>
-      <c r="H27" s="37" t="n">
+      <c r="H27" s="37">
         <v>698</v>
       </c>
-      <c r="I27" s="37" t="n">
+      <c r="I27" s="37">
         <v>746</v>
       </c>
-      <c r="J27" s="37" t="n">
+      <c r="J27" s="37">
         <v>54728</v>
       </c>
-      <c r="K27" s="37" t="n">
+      <c r="K27" s="37">
         <v>50</v>
       </c>
       <c r="L27" s="33">
@@ -2557,120 +2442,116 @@
       </c>
       <c r="N27" s="34">
         <f>100/B27*(F27+J27)</f>
-        <v>35.48135816816911</v>
-      </c>
-      <c r="O27" s="35" t="n">
-        <v>2131.37250427838</v>
-      </c>
-      <c r="P27" s="37" t="n"/>
-      <c r="Q27" s="37" t="n"/>
-      <c r="R27" s="37" t="n"/>
-      <c r="S27" s="38" t="n"/>
-      <c r="T27" s="38" t="n"/>
-      <c r="U27" s="38" t="n"/>
-      <c r="V27" s="40" t="n"/>
-      <c r="W27" s="40" t="n"/>
-      <c r="X27" s="39" t="n"/>
-      <c r="Y27" s="36" t="n"/>
-      <c r="Z27" s="36" t="n"/>
+        <v>35.481358168169109</v>
+      </c>
+      <c r="O27" s="35">
+        <v>2131.3725042783799</v>
+      </c>
+      <c r="P27" s="37"/>
+      <c r="Q27" s="37"/>
+      <c r="R27" s="37"/>
+      <c r="S27" s="38"/>
+      <c r="T27" s="38"/>
+      <c r="U27" s="38"/>
+      <c r="V27" s="40"/>
+      <c r="W27" s="40"/>
+      <c r="X27" s="39"/>
+      <c r="Y27" s="36"/>
+      <c r="Z27" s="36"/>
     </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Taweeq Park</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="4">
         <v>140509</v>
       </c>
-      <c r="C28" s="37" t="n">
+      <c r="C28" s="37">
         <v>61512</v>
       </c>
-      <c r="D28" s="37" t="n">
+      <c r="D28" s="37">
         <v>0</v>
       </c>
-      <c r="E28" s="37" t="n">
+      <c r="E28" s="37">
         <v>0</v>
       </c>
-      <c r="F28" s="37" t="n">
+      <c r="F28" s="37">
         <v>0</v>
       </c>
-      <c r="G28" s="37" t="n">
+      <c r="G28" s="37">
         <v>61512</v>
       </c>
-      <c r="H28" s="37" t="n">
+      <c r="H28" s="37">
         <v>1026</v>
       </c>
-      <c r="I28" s="37" t="n">
+      <c r="I28" s="37">
         <v>1026</v>
       </c>
-      <c r="J28" s="37" t="n">
+      <c r="J28" s="37">
         <v>28963</v>
       </c>
-      <c r="K28" s="37" t="n">
+      <c r="K28" s="37">
         <v>50</v>
       </c>
       <c r="L28" s="33">
         <f>100/B28*E28</f>
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="M28" s="33">
         <f>100/B28*F28</f>
-        <v>0.0</v>
+        <v>0</v>
       </c>
       <c r="N28" s="34">
         <f>100/B28*(F28+J28)</f>
         <v>20.612914475229342</v>
       </c>
-      <c r="O28" s="35" t="n">
-        <v>1277.354545454545</v>
-      </c>
-      <c r="P28" s="37" t="n"/>
-      <c r="Q28" s="37" t="n"/>
-      <c r="R28" s="37" t="n"/>
-      <c r="S28" s="38" t="n"/>
-      <c r="T28" s="38" t="n"/>
-      <c r="U28" s="38" t="n"/>
-      <c r="V28" s="38" t="n"/>
-      <c r="W28" s="38" t="n"/>
-      <c r="X28" s="39" t="n"/>
-      <c r="Y28" s="36" t="n"/>
-      <c r="Z28" s="36" t="n"/>
+      <c r="O28" s="35">
+        <v>1277.3545454545449</v>
+      </c>
+      <c r="P28" s="37"/>
+      <c r="Q28" s="37"/>
+      <c r="R28" s="37"/>
+      <c r="S28" s="38"/>
+      <c r="T28" s="38"/>
+      <c r="U28" s="38"/>
+      <c r="V28" s="38"/>
+      <c r="W28" s="38"/>
+      <c r="X28" s="39"/>
+      <c r="Y28" s="36"/>
+      <c r="Z28" s="36"/>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Bader Park</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="4">
         <v>5120</v>
       </c>
-      <c r="C29" s="37" t="n">
+      <c r="C29" s="37">
         <v>2180</v>
       </c>
-      <c r="D29" s="37" t="n">
+      <c r="D29" s="37">
         <v>19</v>
       </c>
-      <c r="E29" s="37" t="n">
+      <c r="E29" s="37">
         <v>458</v>
       </c>
-      <c r="F29" s="37" t="n">
+      <c r="F29" s="37">
         <v>926</v>
       </c>
-      <c r="G29" s="37" t="n">
+      <c r="G29" s="37">
         <v>1254</v>
       </c>
-      <c r="H29" s="37" t="n">
+      <c r="H29" s="37">
         <v>6</v>
       </c>
-      <c r="I29" s="37" t="n">
+      <c r="I29" s="37">
         <v>25</v>
       </c>
-      <c r="J29" s="37" t="n">
+      <c r="J29" s="37">
         <v>470</v>
       </c>
-      <c r="K29" s="37" t="n">
+      <c r="K29" s="37">
         <v>50</v>
       </c>
       <c r="L29" s="33">
@@ -2685,55 +2566,53 @@
         <f>100/B29*(F29+J29)</f>
         <v>27.265625</v>
       </c>
-      <c r="O29" s="35" t="n">
+      <c r="O29" s="35">
         <v>33.52699784017279</v>
       </c>
-      <c r="P29" s="37" t="n"/>
-      <c r="Q29" s="37" t="n"/>
-      <c r="R29" s="37" t="n"/>
-      <c r="S29" s="38" t="n"/>
-      <c r="T29" s="38" t="n"/>
-      <c r="U29" s="38" t="n"/>
-      <c r="V29" s="38" t="n"/>
-      <c r="W29" s="38" t="n"/>
-      <c r="X29" s="39" t="n"/>
-      <c r="Y29" s="36" t="n"/>
-      <c r="Z29" s="36" t="n"/>
+      <c r="P29" s="37"/>
+      <c r="Q29" s="37"/>
+      <c r="R29" s="37"/>
+      <c r="S29" s="38"/>
+      <c r="T29" s="38"/>
+      <c r="U29" s="38"/>
+      <c r="V29" s="38"/>
+      <c r="W29" s="38"/>
+      <c r="X29" s="39"/>
+      <c r="Y29" s="36"/>
+      <c r="Z29" s="36"/>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Al Arid Park</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="n">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="4">
         <v>63501</v>
       </c>
-      <c r="C30" s="37" t="n">
+      <c r="C30" s="37">
         <v>22552</v>
       </c>
-      <c r="D30" s="37" t="n">
+      <c r="D30" s="37">
         <v>4</v>
       </c>
-      <c r="E30" s="37" t="n">
+      <c r="E30" s="37">
         <v>66</v>
       </c>
-      <c r="F30" s="37" t="n">
+      <c r="F30" s="37">
         <v>179</v>
       </c>
-      <c r="G30" s="37" t="n">
+      <c r="G30" s="37">
         <v>22373</v>
       </c>
-      <c r="H30" s="37" t="n">
+      <c r="H30" s="37">
         <v>185</v>
       </c>
-      <c r="I30" s="37" t="n">
+      <c r="I30" s="37">
         <v>189</v>
       </c>
-      <c r="J30" s="37" t="n">
+      <c r="J30" s="37">
         <v>18523</v>
       </c>
-      <c r="K30" s="37" t="n">
+      <c r="K30" s="37">
         <v>50</v>
       </c>
       <c r="L30" s="33">
@@ -2742,26 +2621,26 @@
       </c>
       <c r="M30" s="33">
         <f>100/B30*F30</f>
-        <v>0.2818853246405569</v>
+        <v>0.28188532464055688</v>
       </c>
       <c r="N30" s="34">
         <f>100/B30*(F30+J30)</f>
         <v>29.451504700713375</v>
       </c>
-      <c r="O30" s="35" t="n">
-        <v>705.5083798882681</v>
-      </c>
-      <c r="P30" s="37" t="n"/>
-      <c r="Q30" s="37" t="n"/>
-      <c r="R30" s="37" t="n"/>
-      <c r="S30" s="38" t="n"/>
-      <c r="T30" s="38" t="n"/>
-      <c r="U30" s="38" t="n"/>
-      <c r="V30" s="38" t="n"/>
-      <c r="W30" s="38" t="n"/>
-      <c r="X30" s="39" t="n"/>
-      <c r="Y30" s="36" t="n"/>
-      <c r="Z30" s="36" t="n"/>
+      <c r="O30" s="35">
+        <v>705.50837988826811</v>
+      </c>
+      <c r="P30" s="37"/>
+      <c r="Q30" s="37"/>
+      <c r="R30" s="37"/>
+      <c r="S30" s="38"/>
+      <c r="T30" s="38"/>
+      <c r="U30" s="38"/>
+      <c r="V30" s="38"/>
+      <c r="W30" s="38"/>
+      <c r="X30" s="39"/>
+      <c r="Y30" s="36"/>
+      <c r="Z30" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2772,7 +2651,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2780,11 +2659,11 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="19" priority="38" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2793,7 +2672,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2801,13 +2680,13 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:L24">
-    <cfRule type="cellIs" priority="24" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="18" priority="24" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2816,7 +2695,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2824,7 +2703,7 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2834,7 +2713,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2842,7 +2721,7 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2852,39 +2731,39 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="17" priority="9" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L26:M30">
-    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="16" priority="6" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3:N17">
-    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="15" priority="37" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L19:N24">
-    <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="14" priority="15" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3:M6">
-    <cfRule type="cellIs" priority="33" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="13" priority="33" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2893,7 +2772,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2901,13 +2780,13 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M8:M17">
-    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="12" priority="32" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2916,7 +2795,7 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2924,13 +2803,13 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M19:M24">
-    <cfRule type="cellIs" priority="14" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="11" priority="14" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2939,7 +2818,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2947,7 +2826,25 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M21 M24">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
+        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
+        <color theme="6" tint="0.59999389629810485"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
+        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2957,7 +2854,7 @@
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -2965,41 +2862,23 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="10" priority="13" operator="lessThan">
       <formula>$K$22</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M21 M24">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
-        <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
-        <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
-        <color rgb="FFFFEF9C"/>
-      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M26:M30">
-    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="formula" val="&quot;M&gt;G&quot;"/>
         <cfvo type="formula" val="&quot;M&lt;G&quot;"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
@@ -3007,47 +2886,47 @@
       <colorScale>
         <cfvo type="formula" val="$M$4:$M$18&gt;$K$4:$K$18"/>
         <cfvo type="formula" val="$M$4:$M$18&lt;$K$4:$K$18"/>
-        <color theme="6" tint="0.5999938962981048"/>
+        <color theme="6" tint="0.59999389629810485"/>
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M29">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="lessThan">
       <formula>$K$33</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N9">
-    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="7" priority="34" operator="lessThan">
       <formula>$K$9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N13">
-    <cfRule type="cellIs" priority="12" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="6" priority="12" operator="greaterThan">
       <formula>$K$13</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N13:N14">
-    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="5" priority="31" operator="lessThan">
       <formula>$K$9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N14">
-    <cfRule type="cellIs" priority="35" operator="equal" dxfId="0">
+    <cfRule type="cellIs" dxfId="4" priority="35" operator="equal">
       <formula>$K$14</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="36" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="3" priority="36" operator="greaterThan">
       <formula>$K$14</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N26:N30">
-    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
       <formula>$K$26</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
       <formula>$K$26</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>